<commit_message>
Rewrite links to migrated pages; add Security page blocks and import
- bradescobank-links transformer: links to migrated pages become
  site-relative (following the source's /en redirects); others stay
  on the original site. Re-imported all migrated pages.
- Security page: cards-note, accordion-tips and columns-image-bleed
  blocks (cards-note and accordion-tips still have structural styling
  only), parsers, import script and template

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-bank-holidays.report.xlsx
+++ b/tools/importer/reports/import-bank-holidays.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-08T17:15:47.276Z</t>
+    <t>2026-10-09T11:27:31.412Z</t>
   </si>
   <si>
     <t>Bradesco Bank</t>
@@ -73,13 +73,97 @@
     <t>bank-holidays</t>
   </si>
   <si>
-    <t>2026-10-09T01:38:04.138Z</t>
+    <t>2026-10-09T11:28:15.670Z</t>
   </si>
   <si>
     <t>Bank Holidays – Bradesco Bank</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/bank-holidays/</t>
+  </si>
+  <si>
+    <t>en/cra-public-file.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-icon"]</t>
+  </si>
+  <si>
+    <t>en/cra-public-file</t>
+  </si>
+  <si>
+    <t>cra-public-file</t>
+  </si>
+  <si>
+    <t>2026-10-09T02:37:20.746Z</t>
+  </si>
+  <si>
+    <t>CRA Public File – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/cra-public-file/</t>
+  </si>
+  <si>
+    <t>en/help.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns-contact"]</t>
+  </si>
+  <si>
+    <t>en/help</t>
+  </si>
+  <si>
+    <t>help</t>
+  </si>
+  <si>
+    <t>2026-10-09T01:53:09.734Z</t>
+  </si>
+  <si>
+    <t>How Can We Help? – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/help/</t>
+  </si>
+  <si>
+    <t>en/other-disclosures.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-download"]</t>
+  </si>
+  <si>
+    <t>en/other-disclosures</t>
+  </si>
+  <si>
+    <t>other-disclosures</t>
+  </si>
+  <si>
+    <t>2026-10-09T02:14:51.356Z</t>
+  </si>
+  <si>
+    <t>Other disclosures – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/other-disclosures/</t>
+  </si>
+  <si>
+    <t>en/security.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-note","cards-note","cards-note","accordion-tips","columns-image-bleed"]</t>
+  </si>
+  <si>
+    <t>en/security</t>
+  </si>
+  <si>
+    <t>security</t>
+  </si>
+  <si>
+    <t>2026-10-09T02:57:45.360Z</t>
+  </si>
+  <si>
+    <t>Security – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/security/</t>
   </si>
 </sst>
 </file>
@@ -468,16 +552,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="31" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -556,6 +640,110 @@
       </c>
       <c r="H3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>